<commit_message>
sprint 2 complete: auto-refresh, session summary, PHAT weeks 3-4, readme updated
</commit_message>
<xml_diff>
--- a/phat_import.xlsx
+++ b/phat_import.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="717" uniqueCount="50">
   <si>
     <t>week</t>
   </si>
@@ -453,7 +453,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B2" s="1">
         <v>1.0</v>
@@ -474,7 +474,7 @@
         <v>2.0</v>
       </c>
       <c r="H2" s="1">
-        <v>0.7</v>
+        <v>0.75</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>11</v>
@@ -482,7 +482,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B3" s="1">
         <v>1.0</v>
@@ -503,7 +503,7 @@
         <v>1.0</v>
       </c>
       <c r="H3" s="1">
-        <v>0.7</v>
+        <v>0.75</v>
       </c>
       <c r="I3" s="1" t="s">
         <v>11</v>
@@ -511,7 +511,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B4" s="1">
         <v>1.0</v>
@@ -532,7 +532,7 @@
         <v>0.0</v>
       </c>
       <c r="H4" s="1">
-        <v>0.7</v>
+        <v>0.75</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>11</v>
@@ -540,7 +540,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B5" s="1">
         <v>1.0</v>
@@ -567,7 +567,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B6" s="1">
         <v>1.0</v>
@@ -594,7 +594,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B7" s="1">
         <v>1.0</v>
@@ -621,7 +621,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B8" s="1">
         <v>1.0</v>
@@ -648,7 +648,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B9" s="1">
         <v>1.0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="10">
       <c r="A10" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B10" s="1">
         <v>1.0</v>
@@ -702,7 +702,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B11" s="1">
         <v>1.0</v>
@@ -729,7 +729,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B12" s="1">
         <v>1.0</v>
@@ -756,7 +756,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B13" s="1">
         <v>1.0</v>
@@ -783,7 +783,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B14" s="1">
         <v>1.0</v>
@@ -810,7 +810,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B15" s="1">
         <v>1.0</v>
@@ -837,7 +837,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B16" s="1">
         <v>1.0</v>
@@ -864,7 +864,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B17" s="1">
         <v>1.0</v>
@@ -891,7 +891,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B18" s="1">
         <v>1.0</v>
@@ -918,7 +918,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B19" s="1">
         <v>1.0</v>
@@ -945,7 +945,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B20" s="1">
         <v>1.0</v>
@@ -972,7 +972,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B21" s="1">
         <v>1.0</v>
@@ -999,7 +999,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B22" s="1">
         <v>1.0</v>
@@ -1026,7 +1026,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B23" s="1">
         <v>2.0</v>
@@ -1047,7 +1047,7 @@
         <v>2.0</v>
       </c>
       <c r="H23" s="1">
-        <v>0.7</v>
+        <v>0.75</v>
       </c>
       <c r="I23" s="1" t="s">
         <v>11</v>
@@ -1055,7 +1055,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B24" s="1">
         <v>2.0</v>
@@ -1076,7 +1076,7 @@
         <v>1.0</v>
       </c>
       <c r="H24" s="1">
-        <v>0.7</v>
+        <v>0.75</v>
       </c>
       <c r="I24" s="1" t="s">
         <v>11</v>
@@ -1084,7 +1084,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B25" s="1">
         <v>2.0</v>
@@ -1105,7 +1105,7 @@
         <v>0.0</v>
       </c>
       <c r="H25" s="1">
-        <v>0.7</v>
+        <v>0.75</v>
       </c>
       <c r="I25" s="1" t="s">
         <v>11</v>
@@ -1113,7 +1113,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B26" s="1">
         <v>2.0</v>
@@ -1140,7 +1140,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B27" s="1">
         <v>2.0</v>
@@ -1167,7 +1167,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B28" s="1">
         <v>2.0</v>
@@ -1194,7 +1194,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B29" s="1">
         <v>2.0</v>
@@ -1221,7 +1221,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B30" s="1">
         <v>2.0</v>
@@ -1248,7 +1248,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B31" s="1">
         <v>2.0</v>
@@ -1275,7 +1275,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B32" s="1">
         <v>2.0</v>
@@ -1302,7 +1302,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B33" s="1">
         <v>2.0</v>
@@ -1329,7 +1329,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B34" s="1">
         <v>2.0</v>
@@ -1356,7 +1356,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B35" s="1">
         <v>2.0</v>
@@ -1383,7 +1383,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B36" s="1">
         <v>2.0</v>
@@ -1410,7 +1410,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B37" s="1">
         <v>2.0</v>
@@ -1437,7 +1437,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B38" s="1">
         <v>2.0</v>
@@ -1464,7 +1464,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B39" s="1">
         <v>2.0</v>
@@ -1491,7 +1491,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B40" s="1">
         <v>3.0</v>
@@ -1512,7 +1512,7 @@
         <v>3.0</v>
       </c>
       <c r="H40" s="1">
-        <v>0.65</v>
+        <v>0.75</v>
       </c>
       <c r="I40" s="1" t="s">
         <v>11</v>
@@ -1520,7 +1520,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B41" s="1">
         <v>3.0</v>
@@ -1541,7 +1541,7 @@
         <v>3.0</v>
       </c>
       <c r="H41" s="1">
-        <v>0.65</v>
+        <v>0.75</v>
       </c>
       <c r="I41" s="1" t="s">
         <v>11</v>
@@ -1549,7 +1549,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B42" s="1">
         <v>3.0</v>
@@ -1570,7 +1570,7 @@
         <v>3.0</v>
       </c>
       <c r="H42" s="1">
-        <v>0.65</v>
+        <v>0.75</v>
       </c>
       <c r="I42" s="1" t="s">
         <v>11</v>
@@ -1578,7 +1578,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B43" s="1">
         <v>3.0</v>
@@ -1599,7 +1599,7 @@
         <v>3.0</v>
       </c>
       <c r="H43" s="1">
-        <v>0.65</v>
+        <v>0.75</v>
       </c>
       <c r="I43" s="1" t="s">
         <v>11</v>
@@ -1607,7 +1607,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B44" s="1">
         <v>3.0</v>
@@ -1628,7 +1628,7 @@
         <v>3.0</v>
       </c>
       <c r="H44" s="1">
-        <v>0.65</v>
+        <v>0.75</v>
       </c>
       <c r="I44" s="1" t="s">
         <v>11</v>
@@ -1636,7 +1636,7 @@
     </row>
     <row r="45">
       <c r="A45" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B45" s="1">
         <v>3.0</v>
@@ -1657,7 +1657,7 @@
         <v>3.0</v>
       </c>
       <c r="H45" s="1">
-        <v>0.65</v>
+        <v>0.75</v>
       </c>
       <c r="I45" s="1" t="s">
         <v>11</v>
@@ -1665,7 +1665,7 @@
     </row>
     <row r="46">
       <c r="A46" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B46" s="1">
         <v>3.0</v>
@@ -1692,7 +1692,7 @@
     </row>
     <row r="47">
       <c r="A47" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B47" s="1">
         <v>3.0</v>
@@ -1719,7 +1719,7 @@
     </row>
     <row r="48">
       <c r="A48" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B48" s="1">
         <v>3.0</v>
@@ -1746,7 +1746,7 @@
     </row>
     <row r="49">
       <c r="A49" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B49" s="1">
         <v>3.0</v>
@@ -1773,7 +1773,7 @@
     </row>
     <row r="50">
       <c r="A50" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B50" s="1">
         <v>3.0</v>
@@ -1800,7 +1800,7 @@
     </row>
     <row r="51">
       <c r="A51" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B51" s="1">
         <v>3.0</v>
@@ -1827,7 +1827,7 @@
     </row>
     <row r="52">
       <c r="A52" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B52" s="1">
         <v>3.0</v>
@@ -1854,7 +1854,7 @@
     </row>
     <row r="53">
       <c r="A53" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B53" s="1">
         <v>3.0</v>
@@ -1881,7 +1881,7 @@
     </row>
     <row r="54">
       <c r="A54" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B54" s="1">
         <v>3.0</v>
@@ -1908,7 +1908,7 @@
     </row>
     <row r="55">
       <c r="A55" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B55" s="1">
         <v>3.0</v>
@@ -1935,7 +1935,7 @@
     </row>
     <row r="56">
       <c r="A56" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B56" s="1">
         <v>3.0</v>
@@ -1962,7 +1962,7 @@
     </row>
     <row r="57">
       <c r="A57" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B57" s="1">
         <v>3.0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="58">
       <c r="A58" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B58" s="1">
         <v>3.0</v>
@@ -2016,7 +2016,7 @@
     </row>
     <row r="59">
       <c r="A59" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B59" s="1">
         <v>3.0</v>
@@ -2043,7 +2043,7 @@
     </row>
     <row r="60">
       <c r="A60" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B60" s="1">
         <v>3.0</v>
@@ -2070,7 +2070,7 @@
     </row>
     <row r="61">
       <c r="A61" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B61" s="1">
         <v>3.0</v>
@@ -2097,7 +2097,7 @@
     </row>
     <row r="62">
       <c r="A62" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B62" s="1">
         <v>3.0</v>
@@ -2124,7 +2124,7 @@
     </row>
     <row r="63">
       <c r="A63" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B63" s="1">
         <v>3.0</v>
@@ -2151,7 +2151,7 @@
     </row>
     <row r="64">
       <c r="A64" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B64" s="1">
         <v>4.0</v>
@@ -2172,7 +2172,7 @@
         <v>3.0</v>
       </c>
       <c r="H64" s="1">
-        <v>0.65</v>
+        <v>0.75</v>
       </c>
       <c r="I64" s="1" t="s">
         <v>11</v>
@@ -2180,7 +2180,7 @@
     </row>
     <row r="65">
       <c r="A65" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B65" s="1">
         <v>4.0</v>
@@ -2201,7 +2201,7 @@
         <v>3.0</v>
       </c>
       <c r="H65" s="1">
-        <v>0.65</v>
+        <v>0.75</v>
       </c>
       <c r="I65" s="1" t="s">
         <v>11</v>
@@ -2209,7 +2209,7 @@
     </row>
     <row r="66">
       <c r="A66" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B66" s="1">
         <v>4.0</v>
@@ -2230,7 +2230,7 @@
         <v>3.0</v>
       </c>
       <c r="H66" s="1">
-        <v>0.65</v>
+        <v>0.75</v>
       </c>
       <c r="I66" s="1" t="s">
         <v>11</v>
@@ -2238,7 +2238,7 @@
     </row>
     <row r="67">
       <c r="A67" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B67" s="1">
         <v>4.0</v>
@@ -2259,7 +2259,7 @@
         <v>3.0</v>
       </c>
       <c r="H67" s="1">
-        <v>0.65</v>
+        <v>0.75</v>
       </c>
       <c r="I67" s="1" t="s">
         <v>11</v>
@@ -2267,7 +2267,7 @@
     </row>
     <row r="68">
       <c r="A68" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B68" s="1">
         <v>4.0</v>
@@ -2288,7 +2288,7 @@
         <v>3.0</v>
       </c>
       <c r="H68" s="1">
-        <v>0.65</v>
+        <v>0.75</v>
       </c>
       <c r="I68" s="1" t="s">
         <v>11</v>
@@ -2296,7 +2296,7 @@
     </row>
     <row r="69">
       <c r="A69" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B69" s="1">
         <v>4.0</v>
@@ -2317,7 +2317,7 @@
         <v>3.0</v>
       </c>
       <c r="H69" s="1">
-        <v>0.65</v>
+        <v>0.75</v>
       </c>
       <c r="I69" s="1" t="s">
         <v>11</v>
@@ -2325,7 +2325,7 @@
     </row>
     <row r="70">
       <c r="A70" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B70" s="1">
         <v>4.0</v>
@@ -2352,7 +2352,7 @@
     </row>
     <row r="71">
       <c r="A71" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B71" s="1">
         <v>4.0</v>
@@ -2379,7 +2379,7 @@
     </row>
     <row r="72">
       <c r="A72" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B72" s="1">
         <v>4.0</v>
@@ -2406,7 +2406,7 @@
     </row>
     <row r="73">
       <c r="A73" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B73" s="1">
         <v>4.0</v>
@@ -2433,7 +2433,7 @@
     </row>
     <row r="74">
       <c r="A74" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B74" s="1">
         <v>4.0</v>
@@ -2460,7 +2460,7 @@
     </row>
     <row r="75">
       <c r="A75" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B75" s="1">
         <v>4.0</v>
@@ -2487,7 +2487,7 @@
     </row>
     <row r="76">
       <c r="A76" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B76" s="1">
         <v>4.0</v>
@@ -2514,7 +2514,7 @@
     </row>
     <row r="77">
       <c r="A77" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B77" s="1">
         <v>4.0</v>
@@ -2541,7 +2541,7 @@
     </row>
     <row r="78">
       <c r="A78" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B78" s="1">
         <v>4.0</v>
@@ -2568,7 +2568,7 @@
     </row>
     <row r="79">
       <c r="A79" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B79" s="1">
         <v>4.0</v>
@@ -2595,7 +2595,7 @@
     </row>
     <row r="80">
       <c r="A80" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B80" s="1">
         <v>4.0</v>
@@ -2622,7 +2622,7 @@
     </row>
     <row r="81">
       <c r="A81" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B81" s="1">
         <v>4.0</v>
@@ -2649,7 +2649,7 @@
     </row>
     <row r="82">
       <c r="A82" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B82" s="1">
         <v>4.0</v>
@@ -2676,7 +2676,7 @@
     </row>
     <row r="83">
       <c r="A83" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B83" s="1">
         <v>4.0</v>
@@ -2703,7 +2703,7 @@
     </row>
     <row r="84">
       <c r="A84" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B84" s="1">
         <v>4.0</v>
@@ -2730,7 +2730,7 @@
     </row>
     <row r="85">
       <c r="A85" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B85" s="1">
         <v>4.0</v>
@@ -2757,7 +2757,7 @@
     </row>
     <row r="86">
       <c r="A86" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B86" s="1">
         <v>4.0</v>
@@ -2784,7 +2784,7 @@
     </row>
     <row r="87">
       <c r="A87" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B87" s="1">
         <v>4.0</v>
@@ -2811,7 +2811,7 @@
     </row>
     <row r="88">
       <c r="A88" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B88" s="1">
         <v>4.0</v>
@@ -2838,7 +2838,7 @@
     </row>
     <row r="89">
       <c r="A89" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B89" s="1">
         <v>4.0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="90">
       <c r="A90" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B90" s="1">
         <v>4.0</v>
@@ -2892,7 +2892,7 @@
     </row>
     <row r="91">
       <c r="A91" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B91" s="1">
         <v>4.0</v>
@@ -2919,7 +2919,7 @@
     </row>
     <row r="92">
       <c r="A92" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B92" s="1">
         <v>5.0</v>
@@ -2939,14 +2939,16 @@
       <c r="G92" s="1">
         <v>3.0</v>
       </c>
-      <c r="H92" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="I92" s="1"/>
+      <c r="H92" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="I92" s="1" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B93" s="1">
         <v>5.0</v>
@@ -2966,14 +2968,16 @@
       <c r="G93" s="1">
         <v>3.0</v>
       </c>
-      <c r="H93" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="I93" s="1"/>
+      <c r="H93" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="I93" s="1" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B94" s="1">
         <v>5.0</v>
@@ -2993,14 +2997,16 @@
       <c r="G94" s="1">
         <v>3.0</v>
       </c>
-      <c r="H94" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="I94" s="1"/>
+      <c r="H94" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="I94" s="1" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B95" s="1">
         <v>5.0</v>
@@ -3020,14 +3026,16 @@
       <c r="G95" s="1">
         <v>3.0</v>
       </c>
-      <c r="H95" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="I95" s="1"/>
+      <c r="H95" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="I95" s="1" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B96" s="1">
         <v>5.0</v>
@@ -3047,14 +3055,16 @@
       <c r="G96" s="1">
         <v>3.0</v>
       </c>
-      <c r="H96" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="I96" s="1"/>
+      <c r="H96" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="I96" s="1" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B97" s="1">
         <v>5.0</v>
@@ -3074,14 +3084,16 @@
       <c r="G97" s="1">
         <v>3.0</v>
       </c>
-      <c r="H97" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="I97" s="1"/>
+      <c r="H97" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="I97" s="1" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B98" s="1">
         <v>5.0</v>
@@ -3108,7 +3120,7 @@
     </row>
     <row r="99">
       <c r="A99" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B99" s="1">
         <v>5.0</v>
@@ -3135,7 +3147,7 @@
     </row>
     <row r="100">
       <c r="A100" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B100" s="1">
         <v>5.0</v>
@@ -3162,7 +3174,7 @@
     </row>
     <row r="101">
       <c r="A101" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B101" s="1">
         <v>5.0</v>
@@ -3189,7 +3201,7 @@
     </row>
     <row r="102">
       <c r="A102" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B102" s="1">
         <v>5.0</v>
@@ -3216,7 +3228,7 @@
     </row>
     <row r="103">
       <c r="A103" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B103" s="1">
         <v>5.0</v>
@@ -3243,7 +3255,7 @@
     </row>
     <row r="104">
       <c r="A104" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B104" s="1">
         <v>5.0</v>
@@ -3270,7 +3282,7 @@
     </row>
     <row r="105">
       <c r="A105" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B105" s="1">
         <v>5.0</v>
@@ -3297,7 +3309,7 @@
     </row>
     <row r="106">
       <c r="A106" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B106" s="1">
         <v>5.0</v>
@@ -3324,7 +3336,7 @@
     </row>
     <row r="107">
       <c r="A107" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B107" s="1">
         <v>5.0</v>
@@ -3351,7 +3363,7 @@
     </row>
     <row r="108">
       <c r="A108" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B108" s="1">
         <v>5.0</v>
@@ -3378,7 +3390,7 @@
     </row>
     <row r="109">
       <c r="A109" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B109" s="1">
         <v>5.0</v>
@@ -3405,7 +3417,7 @@
     </row>
     <row r="110">
       <c r="A110" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B110" s="1">
         <v>5.0</v>
@@ -3432,7 +3444,7 @@
     </row>
     <row r="111">
       <c r="A111" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B111" s="1">
         <v>5.0</v>
@@ -3459,7 +3471,7 @@
     </row>
     <row r="112">
       <c r="A112" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B112" s="1">
         <v>5.0</v>
@@ -3486,7 +3498,7 @@
     </row>
     <row r="113">
       <c r="A113" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B113" s="1">
         <v>5.0</v>
@@ -3513,7 +3525,7 @@
     </row>
     <row r="114">
       <c r="A114" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B114" s="1">
         <v>5.0</v>
@@ -3540,7 +3552,7 @@
     </row>
     <row r="115">
       <c r="A115" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B115" s="1">
         <v>5.0</v>
@@ -3567,7 +3579,7 @@
     </row>
     <row r="116">
       <c r="A116" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B116" s="1">
         <v>5.0</v>
@@ -3594,7 +3606,7 @@
     </row>
     <row r="117">
       <c r="A117" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B117" s="1">
         <v>5.0</v>
@@ -3621,7 +3633,7 @@
     </row>
     <row r="118">
       <c r="A118" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B118" s="1">
         <v>5.0</v>
@@ -3648,7 +3660,7 @@
     </row>
     <row r="119">
       <c r="A119" s="1">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B119" s="1">
         <v>5.0</v>
@@ -3672,6 +3684,3240 @@
         <v>11</v>
       </c>
       <c r="I119" s="1"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B120" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="C120" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D120" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E120" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F120" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="G120" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H120" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="I120" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B121" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="C121" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D121" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E121" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F121" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="G121" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H121" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="I121" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B122" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="C122" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D122" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E122" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="F122" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="G122" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="H122" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="I122" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B123" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="C123" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D123" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E123" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F123" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="G123" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H123" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I123" s="1"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B124" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="C124" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D124" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E124" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F124" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="G124" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H124" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I124" s="1"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B125" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="C125" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D125" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E125" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F125" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="G125" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H125" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I125" s="1"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B126" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="C126" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D126" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E126" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F126" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="G126" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H126" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I126" s="1"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B127" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="C127" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D127" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E127" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F127" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="G127" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H127" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I127" s="1"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B128" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="C128" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D128" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E128" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F128" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="G128" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H128" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I128" s="1"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B129" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="C129" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D129" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E129" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F129" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="G129" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H129" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I129" s="1"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B130" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="C130" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D130" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E130" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F130" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="G130" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H130" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I130" s="1"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B131" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="C131" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D131" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E131" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="F131" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="G131" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="H131" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I131" s="1"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B132" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="C132" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D132" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E132" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F132" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="G132" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H132" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I132" s="1"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B133" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="C133" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D133" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E133" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F133" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="G133" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H133" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I133" s="1"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B134" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="C134" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D134" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E134" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="F134" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="G134" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="H134" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I134" s="1"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B135" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="C135" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D135" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E135" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F135" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="G135" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H135" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I135" s="1"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B136" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="C136" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D136" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E136" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F136" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="G136" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H136" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I136" s="1"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B137" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="C137" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D137" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E137" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="F137" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="G137" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="H137" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I137" s="1"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B138" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="C138" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D138" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E138" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F138" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="G138" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H138" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I138" s="1"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B139" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="C139" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D139" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E139" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F139" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="G139" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H139" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I139" s="1"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B140" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="C140" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D140" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E140" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="F140" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="G140" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="H140" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I140" s="1"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B141" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="C141" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D141" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E141" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F141" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="G141" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H141" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="I141" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B142" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="C142" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D142" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E142" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F142" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="G142" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H142" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="I142" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B143" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="C143" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D143" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E143" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="F143" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="G143" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="H143" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="I143" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B144" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="C144" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D144" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E144" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F144" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="G144" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H144" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I144" s="1"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B145" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="C145" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D145" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E145" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F145" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="G145" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H145" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I145" s="1"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B146" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="C146" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D146" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E146" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F146" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="G146" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H146" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I146" s="1"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B147" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="C147" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D147" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E147" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F147" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="G147" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H147" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I147" s="1"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B148" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="C148" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D148" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E148" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F148" s="1">
+        <v>6.0</v>
+      </c>
+      <c r="G148" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H148" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I148" s="1"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B149" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="C149" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D149" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E149" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F149" s="1">
+        <v>6.0</v>
+      </c>
+      <c r="G149" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H149" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I149" s="1"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B150" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="C150" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D150" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E150" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="F150" s="1">
+        <v>6.0</v>
+      </c>
+      <c r="G150" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="H150" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I150" s="1"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B151" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="C151" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D151" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E151" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F151" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="G151" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H151" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I151" s="1"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B152" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="C152" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D152" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E152" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F152" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="G152" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H152" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I152" s="1"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B153" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="C153" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D153" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E153" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F153" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="G153" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H153" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I153" s="1"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B154" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="C154" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D154" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E154" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F154" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="G154" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H154" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I154" s="1"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B155" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="C155" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D155" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E155" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="F155" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="G155" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="H155" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I155" s="1"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B156" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="C156" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D156" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E156" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F156" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="G156" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H156" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I156" s="1"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B157" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="C157" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D157" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E157" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F157" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="G157" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H157" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I157" s="1"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B158" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="C158" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D158" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E158" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F158" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="G158" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="H158" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="I158" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B159" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="C159" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D159" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E159" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F159" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="G159" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="H159" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="I159" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B160" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="C160" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D160" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E160" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="F160" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="G160" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="H160" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="I160" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B161" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="C161" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D161" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E161" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="F161" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="G161" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="H161" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="I161" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B162" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="C162" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D162" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E162" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="F162" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="G162" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="H162" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="I162" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B163" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="C163" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D163" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E163" s="1">
+        <v>6.0</v>
+      </c>
+      <c r="F163" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="G163" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="H163" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="I163" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B164" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="C164" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D164" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E164" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F164" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="G164" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H164" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I164" s="1"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B165" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="C165" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D165" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E165" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F165" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="G165" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H165" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I165" s="1"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B166" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="C166" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D166" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E166" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="F166" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="G166" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="H166" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I166" s="1"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B167" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="C167" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D167" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E167" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F167" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="G167" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H167" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I167" s="1"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B168" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="C168" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D168" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E168" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F168" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="G168" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H168" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I168" s="1"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B169" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="C169" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D169" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E169" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="F169" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="G169" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="H169" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I169" s="1"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B170" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="C170" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D170" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E170" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F170" s="1">
+        <v>13.0</v>
+      </c>
+      <c r="G170" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H170" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I170" s="1"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B171" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="C171" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D171" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E171" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F171" s="1">
+        <v>13.0</v>
+      </c>
+      <c r="G171" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H171" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I171" s="1"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B172" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="C172" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D172" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E172" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F172" s="1">
+        <v>17.0</v>
+      </c>
+      <c r="G172" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H172" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I172" s="1"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B173" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="C173" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D173" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E173" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F173" s="1">
+        <v>17.0</v>
+      </c>
+      <c r="G173" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H173" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I173" s="1"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B174" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="C174" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D174" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E174" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F174" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="G174" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H174" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I174" s="1"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B175" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="C175" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D175" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E175" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F175" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="G175" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H175" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I175" s="1"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B176" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="C176" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D176" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E176" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="F176" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="G176" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="H176" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I176" s="1"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B177" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="C177" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D177" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E177" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F177" s="1">
+        <v>13.0</v>
+      </c>
+      <c r="G177" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H177" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I177" s="1"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B178" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="C178" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D178" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E178" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F178" s="1">
+        <v>13.0</v>
+      </c>
+      <c r="G178" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H178" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I178" s="1"/>
+    </row>
+    <row r="179">
+      <c r="A179" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B179" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="C179" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D179" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E179" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F179" s="1">
+        <v>15.0</v>
+      </c>
+      <c r="G179" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H179" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I179" s="1"/>
+    </row>
+    <row r="180">
+      <c r="A180" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B180" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="C180" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D180" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E180" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F180" s="1">
+        <v>15.0</v>
+      </c>
+      <c r="G180" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H180" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I180" s="1"/>
+    </row>
+    <row r="181">
+      <c r="A181" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B181" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="C181" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D181" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E181" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="F181" s="1">
+        <v>15.0</v>
+      </c>
+      <c r="G181" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="H181" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I181" s="1"/>
+    </row>
+    <row r="182">
+      <c r="A182" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B182" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="C182" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D182" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E182" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F182" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="G182" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="H182" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="I182" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B183" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="C183" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D183" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E183" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F183" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="G183" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="H183" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="I183" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B184" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="C184" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D184" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E184" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="F184" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="G184" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="H184" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="I184" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B185" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="C185" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D185" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E185" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="F185" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="G185" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="H185" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="I185" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B186" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="C186" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D186" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E186" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="F186" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="G186" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="H186" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="I186" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B187" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="C187" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D187" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E187" s="1">
+        <v>6.0</v>
+      </c>
+      <c r="F187" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="G187" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="H187" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="I187" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B188" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="C188" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D188" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E188" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F188" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="G188" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H188" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I188" s="1"/>
+    </row>
+    <row r="189">
+      <c r="A189" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B189" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="C189" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D189" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E189" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F189" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="G189" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H189" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I189" s="1"/>
+    </row>
+    <row r="190">
+      <c r="A190" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B190" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="C190" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D190" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E190" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="F190" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="G190" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="H190" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I190" s="1"/>
+    </row>
+    <row r="191">
+      <c r="A191" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B191" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="C191" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D191" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E191" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F191" s="1">
+        <v>13.0</v>
+      </c>
+      <c r="G191" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H191" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I191" s="1"/>
+    </row>
+    <row r="192">
+      <c r="A192" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B192" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="C192" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D192" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E192" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F192" s="1">
+        <v>13.0</v>
+      </c>
+      <c r="G192" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H192" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I192" s="1"/>
+    </row>
+    <row r="193">
+      <c r="A193" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B193" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="C193" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D193" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E193" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F193" s="1">
+        <v>17.0</v>
+      </c>
+      <c r="G193" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H193" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I193" s="1"/>
+    </row>
+    <row r="194">
+      <c r="A194" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B194" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="C194" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D194" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E194" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F194" s="1">
+        <v>17.0</v>
+      </c>
+      <c r="G194" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H194" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I194" s="1"/>
+    </row>
+    <row r="195">
+      <c r="A195" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B195" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="C195" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D195" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E195" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="F195" s="1">
+        <v>17.0</v>
+      </c>
+      <c r="G195" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="H195" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I195" s="1"/>
+    </row>
+    <row r="196">
+      <c r="A196" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B196" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="C196" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D196" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E196" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F196" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="G196" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H196" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I196" s="1"/>
+    </row>
+    <row r="197">
+      <c r="A197" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B197" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="C197" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D197" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E197" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F197" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="G197" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H197" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I197" s="1"/>
+    </row>
+    <row r="198">
+      <c r="A198" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B198" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="C198" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D198" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E198" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="F198" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="G198" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="H198" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I198" s="1"/>
+    </row>
+    <row r="199">
+      <c r="A199" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B199" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="C199" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D199" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E199" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F199" s="1">
+        <v>13.0</v>
+      </c>
+      <c r="G199" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H199" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I199" s="1"/>
+    </row>
+    <row r="200">
+      <c r="A200" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B200" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="C200" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D200" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E200" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F200" s="1">
+        <v>13.0</v>
+      </c>
+      <c r="G200" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H200" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I200" s="1"/>
+    </row>
+    <row r="201">
+      <c r="A201" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B201" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="C201" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D201" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E201" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F201" s="1">
+        <v>17.0</v>
+      </c>
+      <c r="G201" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H201" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I201" s="1"/>
+    </row>
+    <row r="202">
+      <c r="A202" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B202" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="C202" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D202" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E202" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F202" s="1">
+        <v>17.0</v>
+      </c>
+      <c r="G202" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H202" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I202" s="1"/>
+    </row>
+    <row r="203">
+      <c r="A203" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B203" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="C203" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D203" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E203" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F203" s="1">
+        <v>12.0</v>
+      </c>
+      <c r="G203" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H203" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I203" s="1"/>
+    </row>
+    <row r="204">
+      <c r="A204" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B204" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="C204" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D204" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E204" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F204" s="1">
+        <v>12.0</v>
+      </c>
+      <c r="G204" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H204" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I204" s="1"/>
+    </row>
+    <row r="205">
+      <c r="A205" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B205" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="C205" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D205" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E205" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="F205" s="1">
+        <v>12.0</v>
+      </c>
+      <c r="G205" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="H205" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I205" s="1"/>
+    </row>
+    <row r="206">
+      <c r="A206" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B206" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="C206" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D206" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E206" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="F206" s="1">
+        <v>12.0</v>
+      </c>
+      <c r="G206" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="H206" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I206" s="1"/>
+    </row>
+    <row r="207">
+      <c r="A207" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B207" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="C207" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D207" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E207" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F207" s="1">
+        <v>17.0</v>
+      </c>
+      <c r="G207" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H207" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I207" s="1"/>
+    </row>
+    <row r="208">
+      <c r="A208" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B208" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="C208" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D208" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E208" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F208" s="1">
+        <v>17.0</v>
+      </c>
+      <c r="G208" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H208" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I208" s="1"/>
+    </row>
+    <row r="209">
+      <c r="A209" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B209" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="C209" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D209" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E209" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="F209" s="1">
+        <v>17.0</v>
+      </c>
+      <c r="G209" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="H209" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I209" s="1"/>
+    </row>
+    <row r="210">
+      <c r="A210" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B210" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="C210" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D210" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E210" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F210" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="G210" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="H210" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="I210" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B211" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="C211" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D211" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E211" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F211" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="G211" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="H211" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="I211" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B212" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="C212" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D212" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E212" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="F212" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="G212" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="H212" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="I212" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B213" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="C213" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D213" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E213" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="F213" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="G213" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="H213" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="I213" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B214" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="C214" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D214" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E214" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="F214" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="G214" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="H214" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="I214" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B215" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="C215" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D215" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E215" s="1">
+        <v>6.0</v>
+      </c>
+      <c r="F215" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="G215" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="H215" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="I215" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B216" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="C216" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D216" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E216" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F216" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="G216" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H216" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I216" s="1"/>
+    </row>
+    <row r="217">
+      <c r="A217" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B217" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="C217" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D217" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E217" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F217" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="G217" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H217" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I217" s="1"/>
+    </row>
+    <row r="218">
+      <c r="A218" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B218" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="C218" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D218" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E218" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="F218" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="G218" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="H218" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I218" s="1"/>
+    </row>
+    <row r="219">
+      <c r="A219" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B219" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="C219" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D219" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E219" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F219" s="1">
+        <v>13.0</v>
+      </c>
+      <c r="G219" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H219" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I219" s="1"/>
+    </row>
+    <row r="220">
+      <c r="A220" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B220" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="C220" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D220" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E220" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F220" s="1">
+        <v>13.0</v>
+      </c>
+      <c r="G220" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H220" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I220" s="1"/>
+    </row>
+    <row r="221">
+      <c r="A221" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B221" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="C221" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D221" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E221" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="F221" s="1">
+        <v>13.0</v>
+      </c>
+      <c r="G221" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="H221" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I221" s="1"/>
+    </row>
+    <row r="222">
+      <c r="A222" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B222" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="C222" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D222" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E222" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F222" s="1">
+        <v>17.0</v>
+      </c>
+      <c r="G222" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H222" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I222" s="1"/>
+    </row>
+    <row r="223">
+      <c r="A223" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B223" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="C223" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D223" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E223" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F223" s="1">
+        <v>17.0</v>
+      </c>
+      <c r="G223" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H223" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I223" s="1"/>
+    </row>
+    <row r="224">
+      <c r="A224" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B224" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="C224" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D224" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E224" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F224" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="G224" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H224" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I224" s="1"/>
+    </row>
+    <row r="225">
+      <c r="A225" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B225" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="C225" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D225" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E225" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F225" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="G225" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H225" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I225" s="1"/>
+    </row>
+    <row r="226">
+      <c r="A226" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B226" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="C226" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D226" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E226" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="F226" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="G226" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="H226" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I226" s="1"/>
+    </row>
+    <row r="227">
+      <c r="A227" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B227" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="C227" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D227" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E227" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F227" s="1">
+        <v>13.0</v>
+      </c>
+      <c r="G227" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H227" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I227" s="1"/>
+    </row>
+    <row r="228">
+      <c r="A228" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B228" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="C228" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D228" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E228" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F228" s="1">
+        <v>13.0</v>
+      </c>
+      <c r="G228" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H228" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I228" s="1"/>
+    </row>
+    <row r="229">
+      <c r="A229" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B229" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="C229" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D229" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E229" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F229" s="1">
+        <v>17.0</v>
+      </c>
+      <c r="G229" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H229" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I229" s="1"/>
+    </row>
+    <row r="230">
+      <c r="A230" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B230" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="C230" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D230" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E230" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F230" s="1">
+        <v>17.0</v>
+      </c>
+      <c r="G230" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H230" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I230" s="1"/>
+    </row>
+    <row r="231">
+      <c r="A231" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B231" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="C231" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D231" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E231" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F231" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="G231" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H231" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I231" s="1"/>
+    </row>
+    <row r="232">
+      <c r="A232" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B232" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="C232" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D232" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E232" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F232" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="G232" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H232" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I232" s="1"/>
+    </row>
+    <row r="233">
+      <c r="A233" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B233" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="C233" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D233" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E233" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="F233" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="G233" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="H233" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I233" s="1"/>
+    </row>
+    <row r="234">
+      <c r="A234" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B234" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="C234" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D234" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E234" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F234" s="1">
+        <v>13.0</v>
+      </c>
+      <c r="G234" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H234" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I234" s="1"/>
+    </row>
+    <row r="235">
+      <c r="A235" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B235" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="C235" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D235" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E235" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F235" s="1">
+        <v>13.0</v>
+      </c>
+      <c r="G235" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H235" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I235" s="1"/>
+    </row>
+    <row r="236">
+      <c r="A236" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B236" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="C236" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D236" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E236" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="F236" s="1">
+        <v>17.0</v>
+      </c>
+      <c r="G236" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H236" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I236" s="1"/>
+    </row>
+    <row r="237">
+      <c r="A237" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B237" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="C237" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D237" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E237" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F237" s="1">
+        <v>17.0</v>
+      </c>
+      <c r="G237" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H237" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I237" s="1"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>

</xml_diff>